<commit_message>
Övertagande: regeltexten säger att duellen också hoppas över
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/F_nätverkskort.xlsx
+++ b/kortdata/F_nätverkskort.xlsx
@@ -3323,7 +3323,7 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Ditt tvångsbud kan inte stoppas — varken med stoppkort eller riskbuffertar. Spelas när du lägger budet.</t>
+          <t>Ditt tvångsbud kan inte stoppas och ingen duell slås: köpet går igenom. Spelas när du lägger budet.</t>
         </is>
       </c>
       <c r="I72" s="2" t="n">
@@ -3362,7 +3362,7 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Ditt tvångsbud kan inte stoppas — varken med stoppkort eller riskbuffertar. Spelas när du lägger budet.</t>
+          <t>Ditt tvångsbud kan inte stoppas och ingen duell slås: köpet går igenom. Spelas när du lägger budet.</t>
         </is>
       </c>
       <c r="I73" s="2" t="n">

</xml_diff>

<commit_message>
Nätverkskortet PK-81 'Kontor blir bostäder' borttaget
Beslut (Niklas): inga kort kostar pengar. Leken har 82 kort; regelboken 9.9 nämner inte
längre konvertering. Tryckfilen för nätverkskorten byggd om.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/F_nätverkskort.xlsx
+++ b/kortdata/F_nätverkskort.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I84"/>
+  <dimension ref="A1:I83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3695,41 +3695,37 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>PK-81</t>
+          <t>PK-82</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>konvertering</t>
+          <t>motbud</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>nar_som_helst</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
+          <t>reaktivt</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr"/>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Kontor blir bostäder</t>
+          <t>Motbud — vi köper er i stället</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Kontoret stod halvtomt. Nu står det kö till lägenheterna.</t>
+          <t>Ni ville köpa oss? Då köper vi er först.</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Betala 5 Mkr: en egen lokal eller ett eget kontor byggs om till hyresrätt och följer bostadsspåret i yieldbanan. DN och energiklass behålls.</t>
+          <t>Stoppa ett tvångsbud mot dig. Du får dessutom köpa en av budgivarens fastigheter till 1,0 × MV (valfritt).</t>
         </is>
       </c>
       <c r="I82" s="2" t="n">
@@ -3738,11 +3734,11 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>PK-82</t>
+          <t>PK-83</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -3758,12 +3754,12 @@
       <c r="E83" s="2" t="inlineStr"/>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Motbud — vi köper er i stället</t>
+          <t>Pac-Man-försvaret</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Ni ville köpa oss? Då köper vi er först.</t>
+          <t>Det bästa försvaret är ett anfall, gärna mot budgivarens bästa hus.</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -3772,45 +3768,6 @@
         </is>
       </c>
       <c r="I83" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="2" t="n">
-        <v>83</v>
-      </c>
-      <c r="B84" s="2" t="inlineStr">
-        <is>
-          <t>PK-83</t>
-        </is>
-      </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>motbud</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr">
-        <is>
-          <t>reaktivt</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr"/>
-      <c r="F84" s="2" t="inlineStr">
-        <is>
-          <t>Pac-Man-försvaret</t>
-        </is>
-      </c>
-      <c r="G84" s="2" t="inlineStr">
-        <is>
-          <t>Det bästa försvaret är ett anfall, gärna mot budgivarens bästa hus.</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>Stoppa ett tvångsbud mot dig. Du får dessutom köpa en av budgivarens fastigheter till 1,0 × MV (valfritt).</t>
-        </is>
-      </c>
-      <c r="I84" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3861,7 +3818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5088,11 +5045,11 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Kontor blir bostäder</t>
+          <t>Motbud — vi köper er i stället</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -5103,29 +5060,14 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Motbud — vi köper er i stället</t>
+          <t>Pac-Man-försvaret</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
-        <is>
-          <t>ej bestämt</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="n">
-        <v>83</v>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>Pac-Man-försvaret</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
         <is>
           <t>ej bestämt</t>
         </is>
@@ -5421,7 +5363,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>83 (kortspecen: 83)</t>
+          <t>82 (kortspecen: 83; PK-81 Kontor blir bostäder borttaget 2026-09-27 – inga kort kostar pengar)</t>
         </is>
       </c>
     </row>

</xml_diff>